<commit_message>
Transformation in variables Germ percentages: sqtr transformed other trait. log transformed
</commit_message>
<xml_diff>
--- a/results/LM  CWM x microclimatic gradients .xlsx
+++ b/results/LM  CWM x microclimatic gradients .xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/light_dark_temperatures_wp/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{DE4A84E0-3523-459E-B8E2-296418150C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1238E9B4-D443-4A85-A54B-BAA1F8F38DE6}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{DE4A84E0-3523-459E-B8E2-296418150C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49B18FF2-9943-4493-9948-2D7C344E47DC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C92F2DC3-8F19-4060-A710-EE89B2D232E3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C92F2DC3-8F19-4060-A710-EE89B2D232E3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="transformed variables" sheetId="2" r:id="rId1"/>
+    <sheet name="original variables" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="64">
   <si>
     <t>CWM</t>
   </si>
@@ -736,6 +737,119 @@
       </rPr>
       <t xml:space="preserve">                              + elevation                -seed production</t>
     </r>
+  </si>
+  <si>
+    <t>Germination percentage (sqrt)</t>
+  </si>
+  <si>
+    <t>log transformed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log transform odds ratio </t>
+  </si>
+  <si>
+    <t>Log transform odds ratio</t>
+  </si>
+  <si>
+    <t>marginal + elevation + height</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>marginal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                     + FDD                  - germ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                    + GDD                  - germ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                  +FDD                 - germ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                    +FDD                     + odds</t>
+    </r>
+  </si>
+  <si>
+    <t>marginal       +elevation      -floral height</t>
+  </si>
+  <si>
+    <t xml:space="preserve">***  +FDD  -seed production    </t>
   </si>
 </sst>
 </file>
@@ -814,17 +928,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -845,6 +958,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1163,6 +1280,437 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06546D05-6A24-4C8D-8B8C-E57A148802A1}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" customWidth="1"/>
+    <col min="10" max="10" width="7.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+    </row>
+    <row r="6" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+    </row>
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="B10:N10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="K11:N11"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="82" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{778B5001-1C87-4BB6-8343-01187C8998AE}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1191,42 +1739,28 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="2"/>
       <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
@@ -1249,198 +1783,198 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3" t="s">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3" t="s">
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="3"/>
+      <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3" t="s">
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3" t="s">
+      <c r="K6" s="2"/>
+      <c r="L6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3" t="s">
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3" t="s">
+      <c r="K8" s="2"/>
+      <c r="L8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
     </row>
     <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="2"/>
+      <c r="B10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
+      <c r="A11" s="2"/>
       <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
@@ -1455,167 +1989,167 @@
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="J12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L12" s="3" t="s">
+      <c r="L12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N12" s="3" t="s">
+      <c r="N12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O12" s="3" t="s">
+      <c r="O12" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3" t="s">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3" t="s">
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="O13" s="3" t="s">
+      <c r="O13" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
+      <c r="D14" s="2"/>
+      <c r="E14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3" t="s">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3" t="s">
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3" t="s">
+      <c r="K14" s="2"/>
+      <c r="L14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M14" s="3" t="s">
+      <c r="M14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
     </row>
     <row r="15" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3" t="s">
+      <c r="D15" s="2"/>
+      <c r="E15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3" t="s">
+      <c r="G15" s="2"/>
+      <c r="H15" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3" t="s">
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3" t="s">
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Community means analysis and results
</commit_message>
<xml_diff>
--- a/results/LM  CWM x microclimatic gradients .xlsx
+++ b/results/LM  CWM x microclimatic gradients .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{DE4A84E0-3523-459E-B8E2-296418150C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49B18FF2-9943-4493-9948-2D7C344E47DC}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{DE4A84E0-3523-459E-B8E2-296418150C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54A941F8-BF05-43CA-BA47-3DAFE6AB4274}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C92F2DC3-8F19-4060-A710-EE89B2D232E3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C92F2DC3-8F19-4060-A710-EE89B2D232E3}"/>
   </bookViews>
   <sheets>
     <sheet name="transformed variables" sheetId="2" r:id="rId1"/>
@@ -937,11 +937,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1310,43 +1310,43 @@
     </row>
     <row r="2" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4" t="s">
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -1418,7 +1418,7 @@
     </row>
     <row r="6" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1427,14 +1427,14 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -1442,50 +1442,50 @@
     </row>
     <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -1508,43 +1508,43 @@
     </row>
     <row r="10" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
     </row>
     <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4" t="s">
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -1614,96 +1614,96 @@
       </c>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>60</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="L15" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N15" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="F16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="K11:N11"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="K3:N3"/>
     <mergeCell ref="B10:N10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="K11:N11"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="82" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -1742,45 +1742,45 @@
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4" t="s">
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -1858,26 +1858,24 @@
     </row>
     <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -1885,54 +1883,56 @@
     </row>
     <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1956,39 +1956,39 @@
     </row>
     <row r="10" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -2066,90 +2066,90 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>39</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-      <c r="L14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
     <row r="15" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="2"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+      <c r="J15" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M15" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="N15" s="2"/>
-      <c r="O15" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+      <c r="O16" s="2" t="s">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>